<commit_message>
Contador de aplicaciones rechazadas y aplicadas
</commit_message>
<xml_diff>
--- a/applications_tracker.xlsx
+++ b/applications_tracker.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$R$184</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$R$259</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,6 +30,9 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -70,11 +73,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -440,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R184"/>
+  <dimension ref="A1:R263"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -9305,8 +9309,3269 @@
         </is>
       </c>
     </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>184</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>NTT Data</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Spain - A Coruña</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Prácticas Ingeniería Informática - Telecomunicaciones</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G185" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>IT internship</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>185</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Airbus</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Spain - Getafe</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>#Discover II 2026-2027 Internship FDT Stress Team</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G186" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>Engineering / Stress team</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>186</v>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Siemens</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Portugal - Porto</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Azure DevOps Trainee (m/f/d)</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G187" s="3" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>Cloud / DevOps / Azure</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>187</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Airbus</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Portugal - Lisbon</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>IT Trainee</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G188" s="3" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>IT Systems</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>188</v>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Capgemini</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Spain - Valencia</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Prácticas en Ciberseguridad</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G189" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>Cybersecurity internship</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>189</v>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Bosch</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Data Engineering Internship (Lakehouse / Databricks)</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G190" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>Data engineering, cloud, Hadoop to Databricks migration</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="n">
+        <v>190</v>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Zurich Insurance</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Trainee Cloud Application Developer - 133025</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>Zurich Careers / iAgora</t>
+        </is>
+      </c>
+      <c r="G191" s="3" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>Application rejected after recruitment process review</t>
+        </is>
+      </c>
+      <c r="O191" t="inlineStr">
+        <is>
+          <t>Cloud Development</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="n">
+        <v>191</v>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Nokia</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Telecommunication Support Trainee - Global Core Network Team</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>iAgora / Job Portal</t>
+        </is>
+      </c>
+      <c r="G192" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>Strong technical telecom role with exposure to cloud and network core systems</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>Portugal (location not specified)</t>
+        </is>
+      </c>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>International / Hybrid</t>
+        </is>
+      </c>
+      <c r="M192" t="inlineStr">
+        <is>
+          <t>['IMS Voice', 'Packet Core', 'Cloud Infrastructure', 'Linux', 'OpenStack', '3GPP', 'VoLTE / VoWiFi / Vo5G']</t>
+        </is>
+      </c>
+      <c r="N192" t="inlineStr">
+        <is>
+          <t>Telecommunications / Cloud / Network Engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="n">
+        <v>192</v>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Siemens</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Romania</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Siemens Talents Hub Internship 2026 - Data Analytics &amp; Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>iAgora / Siemens Careers</t>
+        </is>
+      </c>
+      <c r="G193" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>R&amp;D internship in AI and Data Analytics</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>Brasov / Cluj-Napoca / Bucharest</t>
+        </is>
+      </c>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>AI, Data Analytics, R&amp;D, Machine Learning, Software Prototyping</t>
+        </is>
+      </c>
+      <c r="P193" t="inlineStr">
+        <is>
+          <t>3 months</t>
+        </is>
+      </c>
+      <c r="Q193" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>193</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Novo Nordisk</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>BI, Data &amp; AI Intern - Complaint Insights Team</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>Career Portal / Application Form</t>
+        </is>
+      </c>
+      <c r="G194" s="3" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>BI + AI internship focused on healthcare data analytics</t>
+        </is>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>Bagsværd</t>
+        </is>
+      </c>
+      <c r="O194" t="inlineStr">
+        <is>
+          <t>Business Intelligence, Data Analytics, AI, Power BI</t>
+        </is>
+      </c>
+      <c r="P194" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="Q194" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R194" t="inlineStr">
+        <is>
+          <t>['Power BI', 'Python', 'SQL', 'AI tools']</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>194</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>NTT DATA</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Prácticas Ingeniería Informática - Telecomunicaciones</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>NTT DATA Careers / iAgora</t>
+        </is>
+      </c>
+      <c r="G195" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>Application confirmed by NTT DATA recruitment team via email</t>
+        </is>
+      </c>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>A Coruña</t>
+        </is>
+      </c>
+      <c r="O195" t="inlineStr">
+        <is>
+          <t>Software Development, Telecommunications, IT</t>
+        </is>
+      </c>
+      <c r="Q195" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>195</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>BBVA</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>BECAS BBVA ÁREAS DE TECNOLOGÍA E INNOVACIÓN 2026</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>BBVA Careers</t>
+        </is>
+      </c>
+      <c r="G196" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>Scholarship/internship application confirmed by BBVA recruitment team</t>
+        </is>
+      </c>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>Madrid</t>
+        </is>
+      </c>
+      <c r="O196" t="inlineStr">
+        <is>
+          <t>Technology, Innovation, IT</t>
+        </is>
+      </c>
+      <c r="Q196" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>196</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Natixis</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>IT Trainee | WE WANT YOU 2026 S2</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>Natixis Careers</t>
+        </is>
+      </c>
+      <c r="G197" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>International trainee program focused on IT, software development, data, cybersecurity and analytics</t>
+        </is>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>Porto / Lisbon</t>
+        </is>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="O197" t="inlineStr">
+        <is>
+          <t>IT Trainee Program, Development, Data, Cybersecurity, DevOps</t>
+        </is>
+      </c>
+      <c r="Q197" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>197</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>NTT Data</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Spain - A Coruña</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Prácticas Ingeniería Informática - Telecomunicaciones</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G198" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>IT internship</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>198</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Airbus</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Spain - Getafe</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>#Discover II 2026-2027 Internship FDT Stress Team</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G199" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>Engineering / Stress team</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>199</v>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Siemens</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Portugal - Porto</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Azure DevOps Trainee (m/f/d)</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G200" s="3" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>Cloud / DevOps / Azure</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="n">
+        <v>200</v>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Airbus</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Portugal - Lisbon</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>IT Trainee</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G201" s="3" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>IT Systems</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="n">
+        <v>201</v>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Capgemini</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Spain - Valencia</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Prácticas en Ciberseguridad</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G202" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>Cybersecurity internship</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="n">
+        <v>202</v>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Bosch</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Data Engineering Internship (Lakehouse / Databricks)</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G203" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>Data engineering, cloud, Hadoop to Databricks migration</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="n">
+        <v>203</v>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Zurich Insurance</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Trainee Cloud Application Developer - 133025</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>Zurich Careers / iAgora</t>
+        </is>
+      </c>
+      <c r="G204" s="3" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>Application rejected after recruitment process review</t>
+        </is>
+      </c>
+      <c r="O204" t="inlineStr">
+        <is>
+          <t>Cloud Development</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="n">
+        <v>204</v>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Nokia</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Telecommunication Support Trainee - Global Core Network Team</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>iAgora / Job Portal</t>
+        </is>
+      </c>
+      <c r="G205" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>Strong technical telecom role with exposure to cloud and network core systems</t>
+        </is>
+      </c>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>Portugal (location not specified)</t>
+        </is>
+      </c>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>International / Hybrid</t>
+        </is>
+      </c>
+      <c r="M205" t="inlineStr">
+        <is>
+          <t>['IMS Voice', 'Packet Core', 'Cloud Infrastructure', 'Linux', 'OpenStack', '3GPP', 'VoLTE / VoWiFi / Vo5G']</t>
+        </is>
+      </c>
+      <c r="N205" t="inlineStr">
+        <is>
+          <t>Telecommunications / Cloud / Network Engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="n">
+        <v>205</v>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Siemens</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Romania</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Siemens Talents Hub Internship 2026 - Data Analytics &amp; Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>iAgora / Siemens Careers</t>
+        </is>
+      </c>
+      <c r="G206" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>R&amp;D internship in AI and Data Analytics</t>
+        </is>
+      </c>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>Brasov / Cluj-Napoca / Bucharest</t>
+        </is>
+      </c>
+      <c r="O206" t="inlineStr">
+        <is>
+          <t>AI, Data Analytics, R&amp;D, Machine Learning, Software Prototyping</t>
+        </is>
+      </c>
+      <c r="P206" t="inlineStr">
+        <is>
+          <t>3 months</t>
+        </is>
+      </c>
+      <c r="Q206" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="n">
+        <v>206</v>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Novo Nordisk</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>BI, Data &amp; AI Intern - Complaint Insights Team</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>Career Portal / Application Form</t>
+        </is>
+      </c>
+      <c r="G207" s="3" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>BI + AI internship focused on healthcare data analytics</t>
+        </is>
+      </c>
+      <c r="K207" t="inlineStr">
+        <is>
+          <t>Bagsværd</t>
+        </is>
+      </c>
+      <c r="O207" t="inlineStr">
+        <is>
+          <t>Business Intelligence, Data Analytics, AI, Power BI</t>
+        </is>
+      </c>
+      <c r="P207" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="Q207" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R207" t="inlineStr">
+        <is>
+          <t>['Power BI', 'Python', 'SQL', 'AI tools']</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="n">
+        <v>207</v>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>NTT DATA</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Prácticas Ingeniería Informática - Telecomunicaciones</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>NTT DATA Careers / iAgora</t>
+        </is>
+      </c>
+      <c r="G208" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>Application confirmed by NTT DATA recruitment team via email</t>
+        </is>
+      </c>
+      <c r="K208" t="inlineStr">
+        <is>
+          <t>A Coruña</t>
+        </is>
+      </c>
+      <c r="O208" t="inlineStr">
+        <is>
+          <t>Software Development, Telecommunications, IT</t>
+        </is>
+      </c>
+      <c r="Q208" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="n">
+        <v>208</v>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>BBVA</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>BECAS BBVA ÁREAS DE TECNOLOGÍA E INNOVACIÓN 2026</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>BBVA Careers</t>
+        </is>
+      </c>
+      <c r="G209" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>Scholarship/internship application confirmed by BBVA recruitment team</t>
+        </is>
+      </c>
+      <c r="K209" t="inlineStr">
+        <is>
+          <t>Madrid</t>
+        </is>
+      </c>
+      <c r="O209" t="inlineStr">
+        <is>
+          <t>Technology, Innovation, IT</t>
+        </is>
+      </c>
+      <c r="Q209" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="n">
+        <v>209</v>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Natixis</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>IT Trainee | WE WANT YOU 2026 S2</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>Natixis Careers</t>
+        </is>
+      </c>
+      <c r="G210" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>International trainee program focused on IT, software development, data, cybersecurity and analytics</t>
+        </is>
+      </c>
+      <c r="K210" t="inlineStr">
+        <is>
+          <t>Porto / Lisbon</t>
+        </is>
+      </c>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="O210" t="inlineStr">
+        <is>
+          <t>IT Trainee Program, Development, Data, Cybersecurity, DevOps</t>
+        </is>
+      </c>
+      <c r="Q210" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="n">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="n">
+        <v>211</v>
+      </c>
+      <c r="G212" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="n">
+        <v>212</v>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>NTT Data</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Spain - A Coruña</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Prácticas Ingeniería Informática - Telecomunicaciones</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G213" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>IT internship</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="n">
+        <v>213</v>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Airbus</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Spain - Getafe</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>#Discover II 2026-2027 Internship FDT Stress Team</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G214" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>Engineering / Stress team</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="n">
+        <v>214</v>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Siemens</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Portugal - Porto</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Azure DevOps Trainee (m/f/d)</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G215" s="3" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>Cloud / DevOps / Azure</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="n">
+        <v>215</v>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Airbus</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Portugal - Lisbon</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>IT Trainee</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G216" s="3" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>IT Systems</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="n">
+        <v>216</v>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Capgemini</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Spain - Valencia</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>Prácticas en Ciberseguridad</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G217" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>Cybersecurity internship</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="n">
+        <v>217</v>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Bosch</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Data Engineering Internship (Lakehouse / Databricks)</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G218" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>Data engineering, cloud, Hadoop to Databricks migration</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="n">
+        <v>218</v>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Zurich Insurance</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Trainee Cloud Application Developer - 133025</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>Zurich Careers / iAgora</t>
+        </is>
+      </c>
+      <c r="G219" s="3" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>Application rejected after recruitment process review</t>
+        </is>
+      </c>
+      <c r="O219" t="inlineStr">
+        <is>
+          <t>Cloud Development</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="n">
+        <v>219</v>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Nokia</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Telecommunication Support Trainee - Global Core Network Team</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>iAgora / Job Portal</t>
+        </is>
+      </c>
+      <c r="G220" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>Strong technical telecom role with exposure to cloud and network core systems</t>
+        </is>
+      </c>
+      <c r="K220" t="inlineStr">
+        <is>
+          <t>Portugal (location not specified)</t>
+        </is>
+      </c>
+      <c r="L220" t="inlineStr">
+        <is>
+          <t>International / Hybrid</t>
+        </is>
+      </c>
+      <c r="M220" t="inlineStr">
+        <is>
+          <t>['IMS Voice', 'Packet Core', 'Cloud Infrastructure', 'Linux', 'OpenStack', '3GPP', 'VoLTE / VoWiFi / Vo5G']</t>
+        </is>
+      </c>
+      <c r="N220" t="inlineStr">
+        <is>
+          <t>Telecommunications / Cloud / Network Engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="n">
+        <v>220</v>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Siemens</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>Romania</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>Siemens Talents Hub Internship 2026 - Data Analytics &amp; Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>iAgora / Siemens Careers</t>
+        </is>
+      </c>
+      <c r="G221" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>R&amp;D internship in AI and Data Analytics</t>
+        </is>
+      </c>
+      <c r="K221" t="inlineStr">
+        <is>
+          <t>Brasov / Cluj-Napoca / Bucharest</t>
+        </is>
+      </c>
+      <c r="O221" t="inlineStr">
+        <is>
+          <t>AI, Data Analytics, R&amp;D, Machine Learning, Software Prototyping</t>
+        </is>
+      </c>
+      <c r="P221" t="inlineStr">
+        <is>
+          <t>3 months</t>
+        </is>
+      </c>
+      <c r="Q221" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="n">
+        <v>221</v>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Novo Nordisk</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>BI, Data &amp; AI Intern - Complaint Insights Team</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>Career Portal / Application Form</t>
+        </is>
+      </c>
+      <c r="G222" s="3" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>BI + AI internship focused on healthcare data analytics</t>
+        </is>
+      </c>
+      <c r="K222" t="inlineStr">
+        <is>
+          <t>Bagsværd</t>
+        </is>
+      </c>
+      <c r="O222" t="inlineStr">
+        <is>
+          <t>Business Intelligence, Data Analytics, AI, Power BI</t>
+        </is>
+      </c>
+      <c r="P222" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="Q222" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R222" t="inlineStr">
+        <is>
+          <t>['Power BI', 'Python', 'SQL', 'AI tools']</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="n">
+        <v>222</v>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>NTT DATA</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>Prácticas Ingeniería Informática - Telecomunicaciones</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>NTT DATA Careers / iAgora</t>
+        </is>
+      </c>
+      <c r="G223" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>Application confirmed by NTT DATA recruitment team via email</t>
+        </is>
+      </c>
+      <c r="K223" t="inlineStr">
+        <is>
+          <t>A Coruña</t>
+        </is>
+      </c>
+      <c r="O223" t="inlineStr">
+        <is>
+          <t>Software Development, Telecommunications, IT</t>
+        </is>
+      </c>
+      <c r="Q223" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="n">
+        <v>223</v>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>BBVA</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>BECAS BBVA ÁREAS DE TECNOLOGÍA E INNOVACIÓN 2026</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>BBVA Careers</t>
+        </is>
+      </c>
+      <c r="G224" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>Scholarship/internship application confirmed by BBVA recruitment team</t>
+        </is>
+      </c>
+      <c r="K224" t="inlineStr">
+        <is>
+          <t>Madrid</t>
+        </is>
+      </c>
+      <c r="O224" t="inlineStr">
+        <is>
+          <t>Technology, Innovation, IT</t>
+        </is>
+      </c>
+      <c r="Q224" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="n">
+        <v>224</v>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Natixis</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>IT Trainee | WE WANT YOU 2026 S2</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>Natixis Careers</t>
+        </is>
+      </c>
+      <c r="G225" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>International trainee program focused on IT, software development, data, cybersecurity and analytics</t>
+        </is>
+      </c>
+      <c r="K225" t="inlineStr">
+        <is>
+          <t>Porto / Lisbon</t>
+        </is>
+      </c>
+      <c r="L225" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="O225" t="inlineStr">
+        <is>
+          <t>IT Trainee Program, Development, Data, Cybersecurity, DevOps</t>
+        </is>
+      </c>
+      <c r="Q225" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="n">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="n">
+        <v>226</v>
+      </c>
+      <c r="G227" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="n">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="n">
+        <v>228</v>
+      </c>
+      <c r="G229" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="n">
+        <v>229</v>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>NTT Data</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Spain - A Coruña</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Prácticas Ingeniería Informática - Telecomunicaciones</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G230" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>IT internship</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="n">
+        <v>230</v>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Airbus</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Spain - Getafe</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>#Discover II 2026-2027 Internship FDT Stress Team</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G231" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>Engineering / Stress team</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="n">
+        <v>231</v>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Siemens</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Portugal - Porto</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Azure DevOps Trainee (m/f/d)</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G232" s="3" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>Cloud / DevOps / Azure</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="n">
+        <v>232</v>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Airbus</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Portugal - Lisbon</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>IT Trainee</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G233" s="3" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>IT Systems</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="n">
+        <v>233</v>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Capgemini</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Spain - Valencia</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Prácticas en Ciberseguridad</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G234" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>Cybersecurity internship</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="n">
+        <v>234</v>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Bosch</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Data Engineering Internship (Lakehouse / Databricks)</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G235" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>Data engineering, cloud, Hadoop to Databricks migration</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="n">
+        <v>235</v>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Zurich Insurance</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Trainee Cloud Application Developer - 133025</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>Zurich Careers / iAgora</t>
+        </is>
+      </c>
+      <c r="G236" s="3" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>Application rejected after recruitment process review</t>
+        </is>
+      </c>
+      <c r="O236" t="inlineStr">
+        <is>
+          <t>Cloud Development</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="n">
+        <v>236</v>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Nokia</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Telecommunication Support Trainee - Global Core Network Team</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>iAgora / Job Portal</t>
+        </is>
+      </c>
+      <c r="G237" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>Strong technical telecom role with exposure to cloud and network core systems</t>
+        </is>
+      </c>
+      <c r="K237" t="inlineStr">
+        <is>
+          <t>Portugal (location not specified)</t>
+        </is>
+      </c>
+      <c r="L237" t="inlineStr">
+        <is>
+          <t>International / Hybrid</t>
+        </is>
+      </c>
+      <c r="M237" t="inlineStr">
+        <is>
+          <t>['IMS Voice', 'Packet Core', 'Cloud Infrastructure', 'Linux', 'OpenStack', '3GPP', 'VoLTE / VoWiFi / Vo5G']</t>
+        </is>
+      </c>
+      <c r="N237" t="inlineStr">
+        <is>
+          <t>Telecommunications / Cloud / Network Engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="n">
+        <v>237</v>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Siemens</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Romania</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Siemens Talents Hub Internship 2026 - Data Analytics &amp; Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>iAgora / Siemens Careers</t>
+        </is>
+      </c>
+      <c r="G238" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>R&amp;D internship in AI and Data Analytics</t>
+        </is>
+      </c>
+      <c r="K238" t="inlineStr">
+        <is>
+          <t>Brasov / Cluj-Napoca / Bucharest</t>
+        </is>
+      </c>
+      <c r="O238" t="inlineStr">
+        <is>
+          <t>AI, Data Analytics, R&amp;D, Machine Learning, Software Prototyping</t>
+        </is>
+      </c>
+      <c r="P238" t="inlineStr">
+        <is>
+          <t>3 months</t>
+        </is>
+      </c>
+      <c r="Q238" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="n">
+        <v>238</v>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Novo Nordisk</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>BI, Data &amp; AI Intern - Complaint Insights Team</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>Career Portal / Application Form</t>
+        </is>
+      </c>
+      <c r="G239" s="3" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>BI + AI internship focused on healthcare data analytics</t>
+        </is>
+      </c>
+      <c r="K239" t="inlineStr">
+        <is>
+          <t>Bagsværd</t>
+        </is>
+      </c>
+      <c r="O239" t="inlineStr">
+        <is>
+          <t>Business Intelligence, Data Analytics, AI, Power BI</t>
+        </is>
+      </c>
+      <c r="P239" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="Q239" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R239" t="inlineStr">
+        <is>
+          <t>['Power BI', 'Python', 'SQL', 'AI tools']</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="n">
+        <v>239</v>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>NTT DATA</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Prácticas Ingeniería Informática - Telecomunicaciones</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>NTT DATA Careers / iAgora</t>
+        </is>
+      </c>
+      <c r="G240" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>Application confirmed by NTT DATA recruitment team via email</t>
+        </is>
+      </c>
+      <c r="K240" t="inlineStr">
+        <is>
+          <t>A Coruña</t>
+        </is>
+      </c>
+      <c r="O240" t="inlineStr">
+        <is>
+          <t>Software Development, Telecommunications, IT</t>
+        </is>
+      </c>
+      <c r="Q240" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="n">
+        <v>240</v>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>BBVA</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>BECAS BBVA ÁREAS DE TECNOLOGÍA E INNOVACIÓN 2026</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>BBVA Careers</t>
+        </is>
+      </c>
+      <c r="G241" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>Scholarship/internship application confirmed by BBVA recruitment team</t>
+        </is>
+      </c>
+      <c r="K241" t="inlineStr">
+        <is>
+          <t>Madrid</t>
+        </is>
+      </c>
+      <c r="O241" t="inlineStr">
+        <is>
+          <t>Technology, Innovation, IT</t>
+        </is>
+      </c>
+      <c r="Q241" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="n">
+        <v>241</v>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Natixis</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>IT Trainee | WE WANT YOU 2026 S2</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>Natixis Careers</t>
+        </is>
+      </c>
+      <c r="G242" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>International trainee program focused on IT, software development, data, cybersecurity and analytics</t>
+        </is>
+      </c>
+      <c r="K242" t="inlineStr">
+        <is>
+          <t>Porto / Lisbon</t>
+        </is>
+      </c>
+      <c r="L242" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="O242" t="inlineStr">
+        <is>
+          <t>IT Trainee Program, Development, Data, Cybersecurity, DevOps</t>
+        </is>
+      </c>
+      <c r="Q242" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="n">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="n">
+        <v>243</v>
+      </c>
+      <c r="G244" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="n">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="n">
+        <v>245</v>
+      </c>
+      <c r="G246" t="n">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="n">
+        <v>246</v>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>NTT Data</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Spain - A Coruña</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>Prácticas Ingeniería Informática - Telecomunicaciones</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G247" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>IT internship</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="n">
+        <v>247</v>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Airbus</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Spain - Getafe</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>#Discover II 2026-2027 Internship FDT Stress Team</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G248" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>Engineering / Stress team</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="n">
+        <v>248</v>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Siemens</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>Portugal - Porto</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>Azure DevOps Trainee (m/f/d)</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G249" s="3" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>Cloud / DevOps / Azure</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="n">
+        <v>249</v>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Airbus</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>Portugal - Lisbon</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>IT Trainee</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G250" s="3" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>IT Systems</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="n">
+        <v>250</v>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Capgemini</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>Spain - Valencia</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>Prácticas en Ciberseguridad</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G251" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>Cybersecurity internship</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="n">
+        <v>251</v>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Bosch</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>Data Engineering Internship (Lakehouse / Databricks)</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>iAgora</t>
+        </is>
+      </c>
+      <c r="G252" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>Data engineering, cloud, Hadoop to Databricks migration</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="n">
+        <v>252</v>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Zurich Insurance</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>Trainee Cloud Application Developer - 133025</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>Zurich Careers / iAgora</t>
+        </is>
+      </c>
+      <c r="G253" s="3" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>Application rejected after recruitment process review</t>
+        </is>
+      </c>
+      <c r="O253" t="inlineStr">
+        <is>
+          <t>Cloud Development</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="n">
+        <v>253</v>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Nokia</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Telecommunication Support Trainee - Global Core Network Team</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>iAgora / Job Portal</t>
+        </is>
+      </c>
+      <c r="G254" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>Strong technical telecom role with exposure to cloud and network core systems</t>
+        </is>
+      </c>
+      <c r="K254" t="inlineStr">
+        <is>
+          <t>Portugal (location not specified)</t>
+        </is>
+      </c>
+      <c r="L254" t="inlineStr">
+        <is>
+          <t>International / Hybrid</t>
+        </is>
+      </c>
+      <c r="M254" t="inlineStr">
+        <is>
+          <t>['IMS Voice', 'Packet Core', 'Cloud Infrastructure', 'Linux', 'OpenStack', '3GPP', 'VoLTE / VoWiFi / Vo5G']</t>
+        </is>
+      </c>
+      <c r="N254" t="inlineStr">
+        <is>
+          <t>Telecommunications / Cloud / Network Engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="n">
+        <v>254</v>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Siemens</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Romania</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>Siemens Talents Hub Internship 2026 - Data Analytics &amp; Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>iAgora / Siemens Careers</t>
+        </is>
+      </c>
+      <c r="G255" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>R&amp;D internship in AI and Data Analytics</t>
+        </is>
+      </c>
+      <c r="K255" t="inlineStr">
+        <is>
+          <t>Brasov / Cluj-Napoca / Bucharest</t>
+        </is>
+      </c>
+      <c r="O255" t="inlineStr">
+        <is>
+          <t>AI, Data Analytics, R&amp;D, Machine Learning, Software Prototyping</t>
+        </is>
+      </c>
+      <c r="P255" t="inlineStr">
+        <is>
+          <t>3 months</t>
+        </is>
+      </c>
+      <c r="Q255" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="n">
+        <v>255</v>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Novo Nordisk</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>BI, Data &amp; AI Intern - Complaint Insights Team</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>Career Portal / Application Form</t>
+        </is>
+      </c>
+      <c r="G256" s="3" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>BI + AI internship focused on healthcare data analytics</t>
+        </is>
+      </c>
+      <c r="K256" t="inlineStr">
+        <is>
+          <t>Bagsværd</t>
+        </is>
+      </c>
+      <c r="O256" t="inlineStr">
+        <is>
+          <t>Business Intelligence, Data Analytics, AI, Power BI</t>
+        </is>
+      </c>
+      <c r="P256" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="Q256" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R256" t="inlineStr">
+        <is>
+          <t>['Power BI', 'Python', 'SQL', 'AI tools']</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="n">
+        <v>256</v>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>NTT DATA</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>Prácticas Ingeniería Informática - Telecomunicaciones</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>NTT DATA Careers / iAgora</t>
+        </is>
+      </c>
+      <c r="G257" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>Application confirmed by NTT DATA recruitment team via email</t>
+        </is>
+      </c>
+      <c r="K257" t="inlineStr">
+        <is>
+          <t>A Coruña</t>
+        </is>
+      </c>
+      <c r="O257" t="inlineStr">
+        <is>
+          <t>Software Development, Telecommunications, IT</t>
+        </is>
+      </c>
+      <c r="Q257" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="n">
+        <v>257</v>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>BBVA</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>BECAS BBVA ÁREAS DE TECNOLOGÍA E INNOVACIÓN 2026</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>BBVA Careers</t>
+        </is>
+      </c>
+      <c r="G258" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>Scholarship/internship application confirmed by BBVA recruitment team</t>
+        </is>
+      </c>
+      <c r="K258" t="inlineStr">
+        <is>
+          <t>Madrid</t>
+        </is>
+      </c>
+      <c r="O258" t="inlineStr">
+        <is>
+          <t>Technology, Innovation, IT</t>
+        </is>
+      </c>
+      <c r="Q258" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="n">
+        <v>258</v>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Natixis</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>IT Trainee | WE WANT YOU 2026 S2</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>Natixis Careers</t>
+        </is>
+      </c>
+      <c r="G259" s="2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I259" t="inlineStr">
+        <is>
+          <t>International trainee program focused on IT, software development, data, cybersecurity and analytics</t>
+        </is>
+      </c>
+      <c r="K259" t="inlineStr">
+        <is>
+          <t>Porto / Lisbon</t>
+        </is>
+      </c>
+      <c r="L259" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="O259" t="inlineStr">
+        <is>
+          <t>IT Trainee Program, Development, Data, Cybersecurity, DevOps</t>
+        </is>
+      </c>
+      <c r="Q259" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+    </row>
+    <row r="260"/>
+    <row r="261">
+      <c r="A261" s="4" t="inlineStr">
+        <is>
+          <t>Total Rechazadas:</t>
+        </is>
+      </c>
+      <c r="G261" s="4" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="4" t="inlineStr">
+        <is>
+          <t>Total Aplicadas:</t>
+        </is>
+      </c>
+      <c r="G263" s="4" t="n">
+        <v>180</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:R184"/>
+  <autoFilter ref="A1:R259"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Elimina el resumen viejo y imprime uno actualizado
</commit_message>
<xml_diff>
--- a/applications_tracker.xlsx
+++ b/applications_tracker.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q22"/>
+  <dimension ref="A1:Q24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1177,50 +1177,52 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="16"/>
+    <row r="17"/>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>JOB TRACKER DASHBOARD</t>
         </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Total Applications</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>10</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Total Applications</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="B22" t="n">
+      <c r="B24" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>